<commit_message>
fix: restore site_8023 May xlsx + add empty-download guard to daily_update
- Restores past_data/site_8023/2026-05-01.xlsx from commit 65cc44f
  (all-None data was committed on 2026-05-08 after portal returned empty xlsx)
- daily_update.py now backs up the existing xlsx before deleting it,
  validates the downloaded file (counts rows with non-null gen/hours for
  past dates), and restores the backup + exits 1 if the new file is empty

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/past_data/site_8023/2026-05-01.xlsx
+++ b/past_data/site_8023/2026-05-01.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="68">
   <si>
     <t>No.</t>
   </si>
@@ -35,33 +35,120 @@
     <t>평균</t>
   </si>
   <si>
+    <t>463.2</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
+    <t>4.6</t>
+  </si>
+  <si>
     <t>01일</t>
   </si>
   <si>
+    <t>542.4</t>
+  </si>
+  <si>
+    <t>5.4</t>
+  </si>
+  <si>
     <t>02일</t>
   </si>
   <si>
+    <t>345.6</t>
+  </si>
+  <si>
+    <t>888.0</t>
+  </si>
+  <si>
+    <t>3.5</t>
+  </si>
+  <si>
+    <t>8.9</t>
+  </si>
+  <si>
     <t>03일</t>
   </si>
   <si>
+    <t>100.9</t>
+  </si>
+  <si>
+    <t>988.9</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>9.9</t>
+  </si>
+  <si>
     <t>04일</t>
   </si>
   <si>
+    <t>627.2</t>
+  </si>
+  <si>
+    <t>1616.1</t>
+  </si>
+  <si>
+    <t>6.3</t>
+  </si>
+  <si>
+    <t>16.2</t>
+  </si>
+  <si>
     <t>05일</t>
   </si>
   <si>
+    <t>639.8</t>
+  </si>
+  <si>
+    <t>2255.9</t>
+  </si>
+  <si>
+    <t>6.4</t>
+  </si>
+  <si>
+    <t>22.6</t>
+  </si>
+  <si>
     <t>06일</t>
   </si>
   <si>
+    <t>597.3</t>
+  </si>
+  <si>
+    <t>2853.2</t>
+  </si>
+  <si>
+    <t>6.0</t>
+  </si>
+  <si>
+    <t>28.5</t>
+  </si>
+  <si>
     <t>07일</t>
   </si>
   <si>
+    <t>389.1</t>
+  </si>
+  <si>
+    <t>3242.3</t>
+  </si>
+  <si>
+    <t>3.9</t>
+  </si>
+  <si>
+    <t>32.4</t>
+  </si>
+  <si>
     <t>08일</t>
   </si>
   <si>
+    <t>0.0</t>
+  </si>
+  <si>
     <t>09일</t>
   </si>
   <si>
@@ -126,9 +213,6 @@
   </si>
   <si>
     <t>30일</t>
-  </si>
-  <si>
-    <t>0.0</t>
   </si>
   <si>
     <t>31일</t>
@@ -421,13 +505,17 @@
       <c r="B2" t="s" s="24">
         <v>6</v>
       </c>
-      <c r="C2" s="25"/>
+      <c r="C2" t="s" s="25">
+        <v>7</v>
+      </c>
       <c r="D2" t="s" s="26">
-        <v>7</v>
-      </c>
-      <c r="E2" s="27"/>
+        <v>8</v>
+      </c>
+      <c r="E2" t="s" s="27">
+        <v>9</v>
+      </c>
       <c r="F2" t="s" s="28">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" ht="17.25" customHeight="1">
@@ -435,367 +523,599 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="30">
-        <v>8</v>
-      </c>
-      <c r="C3" s="31"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="34"/>
+        <v>10</v>
+      </c>
+      <c r="C3" t="s" s="31">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s" s="32">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s" s="33">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s" s="34">
+        <v>12</v>
+      </c>
     </row>
     <row r="4" ht="17.25" customHeight="1">
       <c r="A4" t="n" s="1">
         <v>3</v>
       </c>
       <c r="B4" t="s" s="35">
-        <v>9</v>
-      </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="39"/>
+        <v>13</v>
+      </c>
+      <c r="C4" t="s" s="36">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s" s="37">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s" s="38">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s" s="39">
+        <v>17</v>
+      </c>
     </row>
     <row r="5" ht="17.25" customHeight="1">
       <c r="A5" t="n" s="1">
         <v>4</v>
       </c>
       <c r="B5" t="s" s="30">
-        <v>10</v>
-      </c>
-      <c r="C5" s="31"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="34"/>
+        <v>18</v>
+      </c>
+      <c r="C5" t="s" s="31">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s" s="32">
+        <v>20</v>
+      </c>
+      <c r="E5" t="s" s="33">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s" s="34">
+        <v>22</v>
+      </c>
     </row>
     <row r="6" ht="17.25" customHeight="1">
       <c r="A6" t="n" s="1">
         <v>5</v>
       </c>
       <c r="B6" t="s" s="35">
-        <v>11</v>
-      </c>
-      <c r="C6" s="36"/>
-      <c r="D6" s="37"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="39"/>
+        <v>23</v>
+      </c>
+      <c r="C6" t="s" s="36">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s" s="37">
+        <v>25</v>
+      </c>
+      <c r="E6" t="s" s="38">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s" s="39">
+        <v>27</v>
+      </c>
     </row>
     <row r="7" ht="17.25" customHeight="1">
       <c r="A7" t="n" s="1">
         <v>6</v>
       </c>
       <c r="B7" t="s" s="30">
-        <v>12</v>
-      </c>
-      <c r="C7" s="31"/>
-      <c r="D7" s="32"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="34"/>
+        <v>28</v>
+      </c>
+      <c r="C7" t="s" s="31">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s" s="32">
+        <v>30</v>
+      </c>
+      <c r="E7" t="s" s="33">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s" s="34">
+        <v>32</v>
+      </c>
     </row>
     <row r="8" ht="17.25" customHeight="1">
       <c r="A8" t="n" s="1">
         <v>7</v>
       </c>
       <c r="B8" t="s" s="35">
-        <v>13</v>
-      </c>
-      <c r="C8" s="36"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="38"/>
-      <c r="F8" s="39"/>
+        <v>33</v>
+      </c>
+      <c r="C8" t="s" s="36">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s" s="37">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s" s="38">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s" s="39">
+        <v>37</v>
+      </c>
     </row>
     <row r="9" ht="17.25" customHeight="1">
       <c r="A9" t="n" s="1">
         <v>8</v>
       </c>
       <c r="B9" t="s" s="30">
-        <v>14</v>
-      </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="34"/>
+        <v>38</v>
+      </c>
+      <c r="C9" t="s" s="31">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s" s="32">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s" s="33">
+        <v>41</v>
+      </c>
+      <c r="F9" t="s" s="34">
+        <v>42</v>
+      </c>
     </row>
     <row r="10" ht="17.25" customHeight="1">
       <c r="A10" t="n" s="1">
         <v>9</v>
       </c>
       <c r="B10" t="s" s="35">
-        <v>15</v>
-      </c>
-      <c r="C10" s="36"/>
-      <c r="D10" s="37"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="39"/>
+        <v>43</v>
+      </c>
+      <c r="C10" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E10" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" ht="17.25" customHeight="1">
       <c r="A11" t="n" s="1">
         <v>10</v>
       </c>
       <c r="B11" t="s" s="30">
-        <v>16</v>
-      </c>
-      <c r="C11" s="31"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="34"/>
+        <v>45</v>
+      </c>
+      <c r="C11" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F11" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="12" ht="17.25" customHeight="1">
       <c r="A12" t="n" s="1">
         <v>11</v>
       </c>
       <c r="B12" t="s" s="35">
-        <v>17</v>
-      </c>
-      <c r="C12" s="36"/>
-      <c r="D12" s="37"/>
-      <c r="E12" s="38"/>
-      <c r="F12" s="39"/>
+        <v>46</v>
+      </c>
+      <c r="C12" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E12" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F12" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="13" ht="17.25" customHeight="1">
       <c r="A13" t="n" s="1">
         <v>12</v>
       </c>
       <c r="B13" t="s" s="30">
-        <v>18</v>
-      </c>
-      <c r="C13" s="31"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="33"/>
-      <c r="F13" s="34"/>
+        <v>47</v>
+      </c>
+      <c r="C13" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E13" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F13" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="14" ht="17.25" customHeight="1">
       <c r="A14" t="n" s="1">
         <v>13</v>
       </c>
       <c r="B14" t="s" s="35">
-        <v>19</v>
-      </c>
-      <c r="C14" s="36"/>
-      <c r="D14" s="37"/>
-      <c r="E14" s="38"/>
-      <c r="F14" s="39"/>
+        <v>48</v>
+      </c>
+      <c r="C14" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D14" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E14" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F14" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="15" ht="17.25" customHeight="1">
       <c r="A15" t="n" s="1">
         <v>14</v>
       </c>
       <c r="B15" t="s" s="30">
-        <v>20</v>
-      </c>
-      <c r="C15" s="31"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="34"/>
+        <v>49</v>
+      </c>
+      <c r="C15" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D15" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E15" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F15" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="16" ht="17.25" customHeight="1">
       <c r="A16" t="n" s="1">
         <v>15</v>
       </c>
       <c r="B16" t="s" s="35">
-        <v>21</v>
-      </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="37"/>
-      <c r="E16" s="38"/>
-      <c r="F16" s="39"/>
+        <v>50</v>
+      </c>
+      <c r="C16" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D16" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E16" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F16" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="17" ht="17.25" customHeight="1">
       <c r="A17" t="n" s="1">
         <v>16</v>
       </c>
       <c r="B17" t="s" s="30">
-        <v>22</v>
-      </c>
-      <c r="C17" s="31"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="33"/>
-      <c r="F17" s="34"/>
+        <v>51</v>
+      </c>
+      <c r="C17" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E17" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F17" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="18" ht="17.25" customHeight="1">
       <c r="A18" t="n" s="1">
         <v>17</v>
       </c>
       <c r="B18" t="s" s="35">
-        <v>23</v>
-      </c>
-      <c r="C18" s="36"/>
-      <c r="D18" s="37"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
+        <v>52</v>
+      </c>
+      <c r="C18" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E18" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F18" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="19" ht="17.25" customHeight="1">
       <c r="A19" t="n" s="1">
         <v>18</v>
       </c>
       <c r="B19" t="s" s="30">
-        <v>24</v>
-      </c>
-      <c r="C19" s="31"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="34"/>
+        <v>53</v>
+      </c>
+      <c r="C19" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D19" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E19" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F19" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="20" ht="17.25" customHeight="1">
       <c r="A20" t="n" s="1">
         <v>19</v>
       </c>
       <c r="B20" t="s" s="35">
-        <v>25</v>
-      </c>
-      <c r="C20" s="36"/>
-      <c r="D20" s="37"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
+        <v>54</v>
+      </c>
+      <c r="C20" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D20" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E20" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F20" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="21" ht="17.25" customHeight="1">
       <c r="A21" t="n" s="1">
         <v>20</v>
       </c>
       <c r="B21" t="s" s="30">
-        <v>26</v>
-      </c>
-      <c r="C21" s="31"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="34"/>
+        <v>55</v>
+      </c>
+      <c r="C21" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D21" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E21" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F21" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="22" ht="17.25" customHeight="1">
       <c r="A22" t="n" s="1">
         <v>21</v>
       </c>
       <c r="B22" t="s" s="35">
-        <v>27</v>
-      </c>
-      <c r="C22" s="36"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
+        <v>56</v>
+      </c>
+      <c r="C22" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D22" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E22" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F22" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="23" ht="17.25" customHeight="1">
       <c r="A23" t="n" s="1">
         <v>22</v>
       </c>
       <c r="B23" t="s" s="30">
-        <v>28</v>
-      </c>
-      <c r="C23" s="31"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="33"/>
-      <c r="F23" s="34"/>
+        <v>57</v>
+      </c>
+      <c r="C23" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D23" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E23" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F23" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="24" ht="17.25" customHeight="1">
       <c r="A24" t="n" s="1">
         <v>23</v>
       </c>
       <c r="B24" t="s" s="35">
-        <v>29</v>
-      </c>
-      <c r="C24" s="36"/>
-      <c r="D24" s="37"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
+        <v>58</v>
+      </c>
+      <c r="C24" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E24" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F24" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="25" ht="17.25" customHeight="1">
       <c r="A25" t="n" s="1">
         <v>24</v>
       </c>
       <c r="B25" t="s" s="30">
-        <v>30</v>
-      </c>
-      <c r="C25" s="31"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="34"/>
+        <v>59</v>
+      </c>
+      <c r="C25" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D25" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E25" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F25" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="26" ht="17.25" customHeight="1">
       <c r="A26" t="n" s="1">
         <v>25</v>
       </c>
       <c r="B26" t="s" s="35">
-        <v>31</v>
-      </c>
-      <c r="C26" s="36"/>
-      <c r="D26" s="37"/>
-      <c r="E26" s="38"/>
-      <c r="F26" s="39"/>
+        <v>60</v>
+      </c>
+      <c r="C26" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D26" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E26" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F26" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="27" ht="17.25" customHeight="1">
       <c r="A27" t="n" s="1">
         <v>26</v>
       </c>
       <c r="B27" t="s" s="30">
-        <v>32</v>
-      </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="34"/>
+        <v>61</v>
+      </c>
+      <c r="C27" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D27" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E27" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F27" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="28" ht="17.25" customHeight="1">
       <c r="A28" t="n" s="1">
         <v>27</v>
       </c>
       <c r="B28" t="s" s="35">
-        <v>33</v>
-      </c>
-      <c r="C28" s="36"/>
-      <c r="D28" s="37"/>
-      <c r="E28" s="38"/>
-      <c r="F28" s="39"/>
+        <v>62</v>
+      </c>
+      <c r="C28" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D28" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E28" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F28" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="29" ht="17.25" customHeight="1">
       <c r="A29" t="n" s="1">
         <v>28</v>
       </c>
       <c r="B29" t="s" s="30">
-        <v>34</v>
-      </c>
-      <c r="C29" s="31"/>
-      <c r="D29" s="32"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="34"/>
+        <v>63</v>
+      </c>
+      <c r="C29" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D29" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E29" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F29" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="30" ht="17.25" customHeight="1">
       <c r="A30" t="n" s="1">
         <v>29</v>
       </c>
       <c r="B30" t="s" s="35">
-        <v>35</v>
-      </c>
-      <c r="C30" s="36"/>
-      <c r="D30" s="37"/>
-      <c r="E30" s="38"/>
-      <c r="F30" s="39"/>
+        <v>64</v>
+      </c>
+      <c r="C30" t="s" s="36">
+        <v>44</v>
+      </c>
+      <c r="D30" t="s" s="37">
+        <v>44</v>
+      </c>
+      <c r="E30" t="s" s="38">
+        <v>44</v>
+      </c>
+      <c r="F30" t="s" s="39">
+        <v>44</v>
+      </c>
     </row>
     <row r="31" ht="17.25" customHeight="1">
       <c r="A31" t="n" s="1">
         <v>30</v>
       </c>
       <c r="B31" t="s" s="30">
-        <v>36</v>
-      </c>
-      <c r="C31" s="31"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="34"/>
+        <v>65</v>
+      </c>
+      <c r="C31" t="s" s="31">
+        <v>44</v>
+      </c>
+      <c r="D31" t="s" s="32">
+        <v>44</v>
+      </c>
+      <c r="E31" t="s" s="33">
+        <v>44</v>
+      </c>
+      <c r="F31" t="s" s="34">
+        <v>44</v>
+      </c>
     </row>
     <row r="32" ht="17.25" customHeight="1">
       <c r="A32" t="n" s="1">
         <v>31</v>
       </c>
       <c r="B32" t="s" s="35">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="C32" t="s" s="36">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D32" t="s" s="37">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E32" t="s" s="38">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F32" t="s" s="39">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" ht="17.25" customHeight="1">
@@ -803,19 +1123,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s" s="30">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="C33" t="s" s="31">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D33" t="s" s="32">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E33" t="s" s="33">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F33" t="s" s="34">
-        <v>38</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>